<commit_message>
Add MW_RunFromSetup batch macro driven by a 'setup' sheet
Reads a manifest from a worksheet named 'setup' (Worksheet | Range | Cumulative
| SigmaMethod) and runs the analytic risk-emergence analysis for each listed
worksheet, writing a comparison to 'RiskEmergence_Summary' (headline figures +
emergence-by-year pattern). Failing rows are flagged, not fatal. Reuses the
validated MW_Compute. Demo workbook now ships a 'setup' sheet plus a second
(Liability) triangle so the batch produces a multi-row comparison.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
+++ b/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Triangle" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liability" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="setup" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -435,154 +437,147 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>This workbook ships the analytic Merz-Wuthrich (2008) one-year CDR as VBA.</t>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Enable the code (one-time):</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>To enable it (one-time, ~30 seconds):</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. Alt+F11 &gt; File &gt; Import File... &gt; MerzWuthrich.bas   (or paste the code,</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1. Press Alt+F11 to open the VBA editor.</t>
+          <t xml:space="preserve">     omitting the first 'Attribute VB_Name' line).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. File &gt; Import File... and choose MerzWuthrich.bas.</t>
+          <t xml:space="preserve">  2. File &gt; Save As &gt; Excel Macro-Enabled Workbook (*.xlsm).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Close the editor. File &gt; Save As &gt; Excel Macro-Enabled Workbook (*.xlsm).</t>
+          <t xml:space="preserve">  3. Run MW_SelfTest (Alt+F8) - should say PASS.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  4. Run the macro MW_SelfTest (Alt+F8) - it should say PASS.</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Cell functions - point at the VALUE BLOCK only (no labels), e.g. C3:L12:</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Cell functions (UDFs) - point them at the VALUE BLOCK only (no labels):</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =MW_EmergenceFactor(Triangle!C3:L12)   =MW_OneYearSE(...)   =MW_UltimateSE(...)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  =MW_EmergenceFactor(Triangle!C3:L12)</t>
+          <t xml:space="preserve">  Optional: sigmaMethod ("loglinear" default | "mack"), isCumulative (False).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  =MW_OneYearSE(Triangle!C3:L12)</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  =MW_UltimateSE(Triangle!C3:L12)</t>
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Macros (Alt+F8):</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  =MW_TotalReserve(Triangle!C3:L12)</t>
+          <t xml:space="preserve">  MW_Report       - per-AY table + totals + emergence pattern for one triangle.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Optional args: sigmaMethod ("loglinear" default | "mack"), isCumulative (False default).</t>
+          <t xml:space="preserve">  MW_Sensitivity  - leave-one-out outliers for one triangle.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MW_RunFromSetup - BATCH: reads the 'setup' sheet and analyses every listed</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Macros (Alt+F8):</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    worksheet, writing a comparison to 'RiskEmergence_Summary'.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MW_Report      - per-AY table + totals + emergence pattern (to a new sheet).</t>
+          <t xml:space="preserve">  MW_SelfTest     - validates against the GenIns reference.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MW_Sensitivity - leave-one-out: which cells/outliers move the one-year risk.</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MW_SelfTest    - validates against the GenIns reference numbers.</t>
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>The 'setup' sheet (this workbook has an example):</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A: Worksheet (required)  B: Range e.g. C3:L12 (blank = sheet's used range)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Expected result for the GenIns triangle on the 'Triangle' sheet:</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  C: Cumulative Y/N (default N)   D: SigmaMethod (default loglinear)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Emergence factor = 72.7%   One-year SE = 1,774,014   Ultimate SE = 2,441,364</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Reference: the GenIns 'Triangle' sheet gives emergence 72.7%,</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Input rules: a SQUARE block of incremental claims, unobserved lower-right left blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Set isCumulative:=True if your block holds cumulative figures instead.</t>
+          <t xml:space="preserve">  one-year SE 1,774,014, ultimate SE 2,441,364.</t>
         </is>
       </c>
     </row>
@@ -597,23 +592,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GenIns (Taylor-Ashe) incremental claims - value block is C3:L12</t>
+          <t>GenIns incremental - value block C3:L12</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>AY \ DY</t>
+          <t>AY/DY</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
@@ -862,44 +857,356 @@
         <v>344014</v>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>Examples (work after importing the module):</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Emergence factor</t>
-        </is>
-      </c>
-      <c r="D16">
-        <f>MW_EmergenceFactor(C3:L12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>One-year SE</t>
-        </is>
-      </c>
-      <c r="D17">
-        <f>MW_OneYearSE(C3:L12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Ultimate SE</t>
-        </is>
-      </c>
-      <c r="D18">
-        <f>MW_UltimateSE(C3:L12)</f>
-        <v/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Liability incremental - value block C3:L12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>AY/DY</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="J2" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K2" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>7717</v>
+      </c>
+      <c r="D3" t="n">
+        <v>21186</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16163</v>
+      </c>
+      <c r="F3" t="n">
+        <v>19519</v>
+      </c>
+      <c r="G3" t="n">
+        <v>15001</v>
+      </c>
+      <c r="H3" t="n">
+        <v>18012</v>
+      </c>
+      <c r="I3" t="n">
+        <v>12478</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9498</v>
+      </c>
+      <c r="K3" t="n">
+        <v>6874</v>
+      </c>
+      <c r="L3" t="n">
+        <v>5142</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9133</v>
+      </c>
+      <c r="D4" t="n">
+        <v>27150</v>
+      </c>
+      <c r="E4" t="n">
+        <v>20034</v>
+      </c>
+      <c r="F4" t="n">
+        <v>18489</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20261</v>
+      </c>
+      <c r="H4" t="n">
+        <v>9912</v>
+      </c>
+      <c r="I4" t="n">
+        <v>7082</v>
+      </c>
+      <c r="J4" t="n">
+        <v>11276</v>
+      </c>
+      <c r="K4" t="n">
+        <v>3871</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6835</v>
+      </c>
+      <c r="D5" t="n">
+        <v>22437</v>
+      </c>
+      <c r="E5" t="n">
+        <v>18458</v>
+      </c>
+      <c r="F5" t="n">
+        <v>28646</v>
+      </c>
+      <c r="G5" t="n">
+        <v>17759</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10675</v>
+      </c>
+      <c r="I5" t="n">
+        <v>45659</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5509</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>7059</v>
+      </c>
+      <c r="D6" t="n">
+        <v>23055</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20484</v>
+      </c>
+      <c r="F6" t="n">
+        <v>18636</v>
+      </c>
+      <c r="G6" t="n">
+        <v>14425</v>
+      </c>
+      <c r="H6" t="n">
+        <v>9473</v>
+      </c>
+      <c r="I6" t="n">
+        <v>9826</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5131</v>
+      </c>
+      <c r="D7" t="n">
+        <v>15738</v>
+      </c>
+      <c r="E7" t="n">
+        <v>21053</v>
+      </c>
+      <c r="F7" t="n">
+        <v>16755</v>
+      </c>
+      <c r="G7" t="n">
+        <v>20545</v>
+      </c>
+      <c r="H7" t="n">
+        <v>11631</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>5682</v>
+      </c>
+      <c r="D8" t="n">
+        <v>15799</v>
+      </c>
+      <c r="E8" t="n">
+        <v>16696</v>
+      </c>
+      <c r="F8" t="n">
+        <v>19639</v>
+      </c>
+      <c r="G8" t="n">
+        <v>20613</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4204</v>
+      </c>
+      <c r="D9" t="n">
+        <v>9365</v>
+      </c>
+      <c r="E9" t="n">
+        <v>15356</v>
+      </c>
+      <c r="F9" t="n">
+        <v>14629</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3106</v>
+      </c>
+      <c r="D10" t="n">
+        <v>11237</v>
+      </c>
+      <c r="E10" t="n">
+        <v>13301</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3617</v>
+      </c>
+      <c r="D11" t="n">
+        <v>11710</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3157</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cumulative</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>SigmaMethod</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Triangle</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C3:L12</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Liability</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C3:L12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add option to exclude the first development column (long-tail lines)
For lines like GL, the volatile first development column - and the immature
most-recent accident year that has only one data point - can skew the emergence
factor. New exclude_first_dev option drops the first dev step (factor f1 and its
variance) and that one-point latest accident year, while keeping DP1 dollars
folded into DP2. Retained accident years' point ultimates are unchanged; their
SEs shift only via the tail-sigma extrapolation now using one fewer period.

- Python: exclude_first_dev on merz_wuthrich(), sensitivity_oneyear(),
  risk_emergence() (both methods), plus drop_first_dev() helper and --exclude-first-dev CLI.
- VBA: excludeFirstDev arg on MW_Compute + all UDFs; MW_Report/MW_Sensitivity prompt
  for it; MW_RunFromSetup reads a new 'ExcludeFirstDev' column (E) on the setup sheet.
- Demo setup sheet gains column E; READMEs updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
+++ b/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -437,147 +437,119 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Enable the code (one-time):</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Enable: Alt+F11 &gt; Import MerzWuthrich.bas (or paste, dropping the first</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1. Alt+F11 &gt; File &gt; Import File... &gt; MerzWuthrich.bas   (or paste the code,</t>
+          <t>'Attribute VB_Name' line) &gt; Save As .xlsm &gt; run MW_SelfTest (should PASS).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     omitting the first 'Attribute VB_Name' line).</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2. File &gt; Save As &gt; Excel Macro-Enabled Workbook (*.xlsm).</t>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>UDFs (point at the VALUE BLOCK only, e.g. C3:L12):</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Run MW_SelfTest (Alt+F8) - should say PASS.</t>
+          <t xml:space="preserve">  =MW_EmergenceFactor(range, [sigmaMethod], [isCumulative], [excludeFirstDev])</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =MW_OneYearSE / =MW_UltimateSE / =MW_TotalReserve  (same optional args)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Cell functions - point at the VALUE BLOCK only (no labels), e.g. C3:L12:</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  excludeFirstDev=TRUE drops the first development column and the immature</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  =MW_EmergenceFactor(Triangle!C3:L12)   =MW_OneYearSE(...)   =MW_UltimateSE(...)</t>
+          <t xml:space="preserve">  most-recent accident year - useful for long-tail lines like GL.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Optional: sigmaMethod ("loglinear" default | "mack"), isCumulative (False).</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Macros (Alt+F8):</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Macros (Alt+F8):</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MW_Report / MW_Sensitivity - one triangle (they prompt for the options).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MW_Report       - per-AY table + totals + emergence pattern for one triangle.</t>
+          <t xml:space="preserve">  MW_RunFromSetup - BATCH over the 'setup' sheet -&gt; RiskEmergence_Summary.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MW_Sensitivity  - leave-one-out outliers for one triangle.</t>
+          <t xml:space="preserve">  MW_Portfolio    - aggregate the summary into one portfolio factor (asks rho).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MW_RunFromSetup - BATCH: reads the 'setup' sheet and analyses every listed</t>
+          <t xml:space="preserve">  MW_SelfTest     - validates against the GenIns reference.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                    worksheet, writing a comparison to 'RiskEmergence_Summary'.</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MW_SelfTest     - validates against the GenIns reference.</t>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>'setup' sheet columns: A Worksheet | B Range (blank=used range) | C Cumulative</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Y/N | D SigmaMethod (loglinear/mack) | E ExcludeFirstDev Y/N</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>The 'setup' sheet (this workbook has an example):</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A: Worksheet (required)  B: Range e.g. C3:L12 (blank = sheet's used range)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  C: Cumulative Y/N (default N)   D: SigmaMethod (default loglinear)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Reference: the GenIns 'Triangle' sheet gives emergence 72.7%,</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  one-year SE 1,774,014, ultimate SE 2,441,364.</t>
+          <t>Reference (GenIns 'Triangle'): emergence 72.7%, one-year 1,774,014, ult 2,441,364.</t>
         </is>
       </c>
     </row>
@@ -1144,13 +1116,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1174,6 +1147,11 @@
           <t>SigmaMethod</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ExcludeFirstDev</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1191,6 +1169,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1204,6 +1187,11 @@
         </is>
       </c>
       <c r="C3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Pre-build RiskEmergence_Summary sheet; clarify per-development-period emergence
- Demo workbook now ships a pre-built 'RiskEmergence_Summary' sheet with title,
  an explanatory note, and all column labels (incl. EF Yr1.. per-period columns)
  so it is clear where outputs land before running.
- MW_FreshSheet now reuses an existing sheet (clears contents) instead of
  deleting it, so a pre-built/positioned results sheet persists.
- MW_RunFromSetup writes a note distinguishing the aggregate emergence factor
  (one-year/ultimate) from per-development-period emergence (EF Yr columns,
  squares sum to 100%). MW_Report's pattern table relabelled accordingly.
- Regenerated paste-ready .txt (fixed an accidental double-append).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
+++ b/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Triangle" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liability" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="setup" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RiskEmergence_Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +31,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,9 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -439,14 +444,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Enable: Alt+F11 &gt; Import MerzWuthrich.bas (or paste, dropping the first</t>
+          <t>Enable: Alt+F11 &gt; Insert &gt; Module &gt; paste 'Risk Emergence VBA code.txt'</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>'Attribute VB_Name' line) &gt; Save As .xlsm &gt; run MW_SelfTest (should PASS).</t>
+          <t>(or Import MerzWuthrich.bas) &gt; Save As .xlsm &gt; run MW_SelfTest (PASS).</t>
         </is>
       </c>
     </row>
@@ -456,98 +461,108 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>UDFs (point at the VALUE BLOCK only, e.g. C3:L12):</t>
+          <t>To analyse your triangles: fill the 'setup' sheet, then run MW_RunFromSetup.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  =MW_EmergenceFactor(range, [sigmaMethod], [isCumulative], [excludeFirstDev])</t>
+          <t>Results land on the 'RiskEmergence_Summary' sheet (already created here).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  =MW_OneYearSE / =MW_UltimateSE / =MW_TotalReserve  (same optional args)</t>
+          <t>Then run MW_Portfolio to aggregate all LoBs into one number.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  excludeFirstDev=TRUE drops the first development column and the immature</t>
+          <t>For a single triangle: select its value block and run MW_Report.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  most-recent accident year - useful for long-tail lines like GL.</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Outputs you get per triangle:</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Macros (Alt+F8):</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Aggregate emergence factor = one-year SE / ultimate SE.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MW_Report / MW_Sensitivity - one triangle (they prompt for the options).</t>
+          <t xml:space="preserve">  - Per-development-period emergence = EF Yr1, EF Yr2, ... (each = that</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MW_RunFromSetup - BATCH over the 'setup' sheet -&gt; RiskEmergence_Summary.</t>
+          <t xml:space="preserve">    future period's CDR SD / ultimate SD; their squares sum to 100%).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MW_Portfolio    - aggregate the summary into one portfolio factor (asks rho).</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MW_SelfTest     - validates against the GenIns reference.</t>
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>UDFs (point at the VALUE BLOCK only, e.g. C3:L12):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =MW_EmergenceFactor(range, [sigmaMethod], [isCumulative], [excludeFirstDev])</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>'setup' sheet columns: A Worksheet | B Range (blank=used range) | C Cumulative</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =MW_OneYearSE / =MW_UltimateSE / =MW_TotalReserve  (same optional args)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Y/N | D SigmaMethod (loglinear/mack) | E ExcludeFirstDev Y/N</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>'setup' columns: A Worksheet | B Range (blank=used range) | C Cumulative Y/N</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  | D SigmaMethod (loglinear/mack) | E ExcludeFirstDev Y/N</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Reference (GenIns 'Triangle'): emergence 72.7%, one-year 1,774,014, ult 2,441,364.</t>
         </is>
@@ -1200,4 +1215,154 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Risk emergence (analytic Merz-Wuthrich) - batch from 'setup'</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aggregate = One-year SE / Ultimate SE (col F). Per-development-period emergence = EF Yr columns (each = that future period's CDR SD / Ultimate SD; squares sum to 100%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Size n</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Total reserve</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Ultimate SE</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>One-year SE</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Emergence factor</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr1</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr2</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr3</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr4</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr5</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr6</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr7</t>
+        </is>
+      </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr8</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t>EF Yr9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Triangle</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(run MW_RunFromSetup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Liability</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(run MW_RunFromSetup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio (after MW_Portfolio)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Surface per-development-period sigma_j; clarify EF Yr1 = aggregate factor
- MW_Report now lists a "Development parameters" block (Dev period, chain-ladder
  factor f_j, Mack's sigma_j). MWResult carries devFactor()/sigma(); Python
  merz_wuthrich() returns a dev_parameters table too.
- Clarified (note on RiskEmergence_Summary): the aggregate emergence factor
  equals EF Yr1 by definition (both = one-year SE / ultimate SE) - not a bug,
  and not sigma_1.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
+++ b/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
@@ -438,9 +438,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -455,9 +453,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -486,9 +482,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
@@ -517,9 +511,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
@@ -541,9 +533,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -558,9 +548,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -1245,7 +1233,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aggregate = One-year SE / Ultimate SE (col F). Per-development-period emergence = EF Yr columns (each = that future period's CDR SD / Ultimate SD; squares sum to 100%).</t>
+          <t>Aggregate emergence factor (col F) = One-year SE / Ultimate SE = EF Yr1 by definition. EF Yr columns = per-development-period emergence (each = that future period's CDR SD / Ultimate SD; squares sum to 100%).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Demo workbook: reserve rows 2-3 for the per-year emergence/reserve strips
Triangle and Liability sheets now start at C5:L14 (headers row 4), with
labelled placeholder rows 2-3 that MW_RunFromSetup fills in place - no row
insertion needed on first run. Setup ranges and ReadMe updated to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
+++ b/Reserve_Risk/vba/MerzWuthrich_demo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -438,7 +438,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -453,7 +452,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -482,7 +480,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
@@ -511,46 +508,57 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - On each triangle sheet itself: row 2 = risk emergence per future year,</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>UDFs (point at the VALUE BLOCK only, e.g. C3:L12):</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    row 3 = remaining reserve at the start of that year (volume weights).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>UDFs (point at the VALUE BLOCK only, e.g. C5:L14):</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t xml:space="preserve">  =MW_EmergenceFactor(range, [sigmaMethod], [isCumulative], [excludeFirstDev])</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  =MW_OneYearSE / =MW_UltimateSE / =MW_TotalReserve  (same optional args)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t xml:space="preserve">  =MW_OneYearSE / =MW_UltimateSE / =MW_TotalReserve  (same optional args)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>'setup' columns: A Worksheet | B Range (blank=used range) | C Cumulative Y/N</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  | D SigmaMethod (loglinear/mack) | E ExcludeFirstDev Y/N</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  | D SigmaMethod (loglinear/mack) | E ExcludeFirstDev Y/N</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Reference (GenIns 'Triangle'): emergence 72.7%, one-year 1,774,014, ult 2,441,364.</t>
         </is>
@@ -567,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -576,259 +584,278 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GenIns incremental - value block C3:L12</t>
+          <t>GenIns incremental - value block C5:L14</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Risk emergence by future year (Yr1, Yr2, ...):</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>(run MW_RunFromSetup to fill rows 2-3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Remaining reserve at start of year:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>AY/DY</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="H4" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="I4" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J4" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K4" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="L2" s="1" t="n">
+      <c r="L4" s="1" t="n">
         <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>357848</v>
-      </c>
-      <c r="D3" t="n">
-        <v>766940</v>
-      </c>
-      <c r="E3" t="n">
-        <v>610542</v>
-      </c>
-      <c r="F3" t="n">
-        <v>482940</v>
-      </c>
-      <c r="G3" t="n">
-        <v>527326</v>
-      </c>
-      <c r="H3" t="n">
-        <v>574398</v>
-      </c>
-      <c r="I3" t="n">
-        <v>146342</v>
-      </c>
-      <c r="J3" t="n">
-        <v>139950</v>
-      </c>
-      <c r="K3" t="n">
-        <v>227229</v>
-      </c>
-      <c r="L3" t="n">
-        <v>67948</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" t="n">
-        <v>352118</v>
-      </c>
-      <c r="D4" t="n">
-        <v>884021</v>
-      </c>
-      <c r="E4" t="n">
-        <v>933894</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1183289</v>
-      </c>
-      <c r="G4" t="n">
-        <v>445745</v>
-      </c>
-      <c r="H4" t="n">
-        <v>320996</v>
-      </c>
-      <c r="I4" t="n">
-        <v>527804</v>
-      </c>
-      <c r="J4" t="n">
-        <v>266172</v>
-      </c>
-      <c r="K4" t="n">
-        <v>425046</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="1" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>290507</v>
+        <v>357848</v>
       </c>
       <c r="D5" t="n">
-        <v>1001799</v>
+        <v>766940</v>
       </c>
       <c r="E5" t="n">
-        <v>926219</v>
+        <v>610542</v>
       </c>
       <c r="F5" t="n">
-        <v>1016654</v>
+        <v>482940</v>
       </c>
       <c r="G5" t="n">
-        <v>750816</v>
+        <v>527326</v>
       </c>
       <c r="H5" t="n">
-        <v>146923</v>
+        <v>574398</v>
       </c>
       <c r="I5" t="n">
-        <v>495992</v>
+        <v>146342</v>
       </c>
       <c r="J5" t="n">
-        <v>280405</v>
+        <v>139950</v>
+      </c>
+      <c r="K5" t="n">
+        <v>227229</v>
+      </c>
+      <c r="L5" t="n">
+        <v>67948</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="1" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>310608</v>
+        <v>352118</v>
       </c>
       <c r="D6" t="n">
-        <v>1108250</v>
+        <v>884021</v>
       </c>
       <c r="E6" t="n">
-        <v>776189</v>
+        <v>933894</v>
       </c>
       <c r="F6" t="n">
-        <v>1562400</v>
+        <v>1183289</v>
       </c>
       <c r="G6" t="n">
-        <v>272482</v>
+        <v>445745</v>
       </c>
       <c r="H6" t="n">
-        <v>352053</v>
+        <v>320996</v>
       </c>
       <c r="I6" t="n">
-        <v>206286</v>
+        <v>527804</v>
+      </c>
+      <c r="J6" t="n">
+        <v>266172</v>
+      </c>
+      <c r="K6" t="n">
+        <v>425046</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="1" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>443160</v>
+        <v>290507</v>
       </c>
       <c r="D7" t="n">
-        <v>693190</v>
+        <v>1001799</v>
       </c>
       <c r="E7" t="n">
-        <v>991983</v>
+        <v>926219</v>
       </c>
       <c r="F7" t="n">
-        <v>769488</v>
+        <v>1016654</v>
       </c>
       <c r="G7" t="n">
-        <v>504851</v>
+        <v>750816</v>
       </c>
       <c r="H7" t="n">
-        <v>470639</v>
+        <v>146923</v>
+      </c>
+      <c r="I7" t="n">
+        <v>495992</v>
+      </c>
+      <c r="J7" t="n">
+        <v>280405</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="1" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>396132</v>
+        <v>310608</v>
       </c>
       <c r="D8" t="n">
-        <v>937085</v>
+        <v>1108250</v>
       </c>
       <c r="E8" t="n">
-        <v>847498</v>
+        <v>776189</v>
       </c>
       <c r="F8" t="n">
-        <v>805037</v>
+        <v>1562400</v>
       </c>
       <c r="G8" t="n">
-        <v>705960</v>
+        <v>272482</v>
+      </c>
+      <c r="H8" t="n">
+        <v>352053</v>
+      </c>
+      <c r="I8" t="n">
+        <v>206286</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="1" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>440832</v>
+        <v>443160</v>
       </c>
       <c r="D9" t="n">
-        <v>847631</v>
+        <v>693190</v>
       </c>
       <c r="E9" t="n">
-        <v>1131398</v>
+        <v>991983</v>
       </c>
       <c r="F9" t="n">
-        <v>1063269</v>
+        <v>769488</v>
+      </c>
+      <c r="G9" t="n">
+        <v>504851</v>
+      </c>
+      <c r="H9" t="n">
+        <v>470639</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="1" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C10" t="n">
-        <v>359480</v>
+        <v>396132</v>
       </c>
       <c r="D10" t="n">
-        <v>1061648</v>
+        <v>937085</v>
       </c>
       <c r="E10" t="n">
-        <v>1443370</v>
+        <v>847498</v>
+      </c>
+      <c r="F10" t="n">
+        <v>805037</v>
+      </c>
+      <c r="G10" t="n">
+        <v>705960</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="1" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C11" t="n">
-        <v>376686</v>
+        <v>440832</v>
       </c>
       <c r="D11" t="n">
-        <v>986608</v>
+        <v>847631</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1131398</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1063269</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>359480</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1061648</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1443370</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" t="n">
+        <v>376686</v>
+      </c>
+      <c r="D13" t="n">
+        <v>986608</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C14" t="n">
         <v>344014</v>
       </c>
     </row>
@@ -843,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -852,259 +879,278 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Liability incremental - value block C3:L12</t>
+          <t>Liability incremental - value block C5:L14</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Risk emergence by future year (Yr1, Yr2, ...):</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>(run MW_RunFromSetup to fill rows 2-3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Remaining reserve at start of year:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>AY/DY</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="H4" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="I4" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J4" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K4" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="L2" s="1" t="n">
+      <c r="L4" s="1" t="n">
         <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>7717</v>
-      </c>
-      <c r="D3" t="n">
-        <v>21186</v>
-      </c>
-      <c r="E3" t="n">
-        <v>16163</v>
-      </c>
-      <c r="F3" t="n">
-        <v>19519</v>
-      </c>
-      <c r="G3" t="n">
-        <v>15001</v>
-      </c>
-      <c r="H3" t="n">
-        <v>18012</v>
-      </c>
-      <c r="I3" t="n">
-        <v>12478</v>
-      </c>
-      <c r="J3" t="n">
-        <v>9498</v>
-      </c>
-      <c r="K3" t="n">
-        <v>6874</v>
-      </c>
-      <c r="L3" t="n">
-        <v>5142</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" t="n">
-        <v>9133</v>
-      </c>
-      <c r="D4" t="n">
-        <v>27150</v>
-      </c>
-      <c r="E4" t="n">
-        <v>20034</v>
-      </c>
-      <c r="F4" t="n">
-        <v>18489</v>
-      </c>
-      <c r="G4" t="n">
-        <v>20261</v>
-      </c>
-      <c r="H4" t="n">
-        <v>9912</v>
-      </c>
-      <c r="I4" t="n">
-        <v>7082</v>
-      </c>
-      <c r="J4" t="n">
-        <v>11276</v>
-      </c>
-      <c r="K4" t="n">
-        <v>3871</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="1" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>6835</v>
+        <v>7717</v>
       </c>
       <c r="D5" t="n">
-        <v>22437</v>
+        <v>21186</v>
       </c>
       <c r="E5" t="n">
-        <v>18458</v>
+        <v>16163</v>
       </c>
       <c r="F5" t="n">
-        <v>28646</v>
+        <v>19519</v>
       </c>
       <c r="G5" t="n">
-        <v>17759</v>
+        <v>15001</v>
       </c>
       <c r="H5" t="n">
-        <v>10675</v>
+        <v>18012</v>
       </c>
       <c r="I5" t="n">
-        <v>45659</v>
+        <v>12478</v>
       </c>
       <c r="J5" t="n">
-        <v>5509</v>
+        <v>9498</v>
+      </c>
+      <c r="K5" t="n">
+        <v>6874</v>
+      </c>
+      <c r="L5" t="n">
+        <v>5142</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="1" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>7059</v>
+        <v>9133</v>
       </c>
       <c r="D6" t="n">
-        <v>23055</v>
+        <v>27150</v>
       </c>
       <c r="E6" t="n">
-        <v>20484</v>
+        <v>20034</v>
       </c>
       <c r="F6" t="n">
-        <v>18636</v>
+        <v>18489</v>
       </c>
       <c r="G6" t="n">
-        <v>14425</v>
+        <v>20261</v>
       </c>
       <c r="H6" t="n">
-        <v>9473</v>
+        <v>9912</v>
       </c>
       <c r="I6" t="n">
-        <v>9826</v>
+        <v>7082</v>
+      </c>
+      <c r="J6" t="n">
+        <v>11276</v>
+      </c>
+      <c r="K6" t="n">
+        <v>3871</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="1" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>5131</v>
+        <v>6835</v>
       </c>
       <c r="D7" t="n">
-        <v>15738</v>
+        <v>22437</v>
       </c>
       <c r="E7" t="n">
-        <v>21053</v>
+        <v>18458</v>
       </c>
       <c r="F7" t="n">
-        <v>16755</v>
+        <v>28646</v>
       </c>
       <c r="G7" t="n">
-        <v>20545</v>
+        <v>17759</v>
       </c>
       <c r="H7" t="n">
-        <v>11631</v>
+        <v>10675</v>
+      </c>
+      <c r="I7" t="n">
+        <v>45659</v>
+      </c>
+      <c r="J7" t="n">
+        <v>5509</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="1" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>5682</v>
+        <v>7059</v>
       </c>
       <c r="D8" t="n">
-        <v>15799</v>
+        <v>23055</v>
       </c>
       <c r="E8" t="n">
-        <v>16696</v>
+        <v>20484</v>
       </c>
       <c r="F8" t="n">
-        <v>19639</v>
+        <v>18636</v>
       </c>
       <c r="G8" t="n">
-        <v>20613</v>
+        <v>14425</v>
+      </c>
+      <c r="H8" t="n">
+        <v>9473</v>
+      </c>
+      <c r="I8" t="n">
+        <v>9826</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="1" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>4204</v>
+        <v>5131</v>
       </c>
       <c r="D9" t="n">
-        <v>9365</v>
+        <v>15738</v>
       </c>
       <c r="E9" t="n">
-        <v>15356</v>
+        <v>21053</v>
       </c>
       <c r="F9" t="n">
-        <v>14629</v>
+        <v>16755</v>
+      </c>
+      <c r="G9" t="n">
+        <v>20545</v>
+      </c>
+      <c r="H9" t="n">
+        <v>11631</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="1" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C10" t="n">
-        <v>3106</v>
+        <v>5682</v>
       </c>
       <c r="D10" t="n">
-        <v>11237</v>
+        <v>15799</v>
       </c>
       <c r="E10" t="n">
-        <v>13301</v>
+        <v>16696</v>
+      </c>
+      <c r="F10" t="n">
+        <v>19639</v>
+      </c>
+      <c r="G10" t="n">
+        <v>20613</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="1" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C11" t="n">
-        <v>3617</v>
+        <v>4204</v>
       </c>
       <c r="D11" t="n">
-        <v>11710</v>
+        <v>9365</v>
+      </c>
+      <c r="E11" t="n">
+        <v>15356</v>
+      </c>
+      <c r="F11" t="n">
+        <v>14629</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3106</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11237</v>
+      </c>
+      <c r="E12" t="n">
+        <v>13301</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3617</v>
+      </c>
+      <c r="D13" t="n">
+        <v>11710</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C14" t="n">
         <v>3157</v>
       </c>
     </row>
@@ -1164,7 +1210,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C3:L12</t>
+          <t>C5:L14</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1186,7 +1232,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C3:L12</t>
+          <t>C5:L14</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>